<commit_message>
Strip em-dashes from all deliverables; add CLAUDE.md copy-style rule
- Removed em-dashes from all build scripts and regenerated every .docx/.xlsx (replaced with commas/periods/colons; en-dashes in numeric ranges kept)
- Added CLAUDE.md: never use em-dashes; no fabricated proof; build-script workflow notes
</commit_message>
<xml_diff>
--- a/Well-and-Good-Websites-Copy-Recommendations-Tracker.xlsx
+++ b/Well-and-Good-Websites-Copy-Recommendations-Tracker.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Get found by local customers — and chosen before the competitor down the street. Live in 24 hours.</t>
+          <t>Get found by local customers, and chosen before the competitor down the street. Live in 24 hours.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Hero H1 — test variant A</t>
+          <t>Hero H1, test variant A</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Get found on Google and chosen by local customers — your site live in 24 hours.</t>
+          <t>Get found on Google and chosen by local customers, your site live in 24 hours.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Hero H1 — test variant B</t>
+          <t>Hero H1, test variant B</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Hero H1 — test variant C</t>
+          <t>Hero H1, test variant C</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>See your new website before you pay a cent — live in 24 hours.</t>
+          <t>See your new website before you pay a cent, live in 24 hours.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[CONFIRM actual button label — not readable from page]</t>
+          <t>[CONFIRM actual button label, not readable from page]</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>See a free preview of your site — no commitment.</t>
+          <t>See a free preview of your site, no commitment.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Everything agencies sell you separately — website, SEO, social, reviews — in one monthly price from $99.</t>
+          <t>Everything agencies sell you separately, website, SEO, social, reviews, in one monthly price from $99.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Frank testimonial — label</t>
+          <t>Frank testimonial, label</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Honest, consistent detail (testimonial wording itself is strong — leave it).</t>
+          <t>Honest, consistent detail (testimonial wording itself is strong, leave it).</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>None — no testimonial, no founder block, no proof (homepage has all three).</t>
+          <t>None, no testimonial, no founder block, no proof (homepage has all three).</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[CONFIRM — may be "When a one-page website works well."]</t>
+          <t>[CONFIRM, may be "When a one-page website works well."]</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Form only — "Tell me about your business and I'll build you a free preview" (you reply later).</t>
+          <t>Form only, "Tell me about your business and I'll build you a free preview" (you reply later).</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">, </t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">, </t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">, </t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">, </t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">, </t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">, </t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t xml:space="preserve">, </t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -1764,28 +1764,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  OPEN — proposed, not yet done. Your action.</t>
+          <t xml:space="preserve"> OPEN, proposed, not yet done. Your action.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  TEST — an A/B variant to try, not a straight swap.</t>
+          <t xml:space="preserve"> TEST, an A/B variant to try, not a straight swap.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  VERIFY — confirm current state on the live site (I couldn't read it).</t>
+          <t xml:space="preserve"> VERIFY, confirm current state on the live site (I couldn't read it).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SHIPPED — already live; shown so you can see progress.</t>
+          <t xml:space="preserve"> SHIPPED, already live; shown so you can see progress.</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Add a 'Notes' or 'Decision' column on the right as you review — yours to edit.</t>
+          <t>Add a 'Notes' or 'Decision' column on the right as you review, yours to edit.</t>
         </is>
       </c>
     </row>

</xml_diff>